<commit_message>
Corrigir nome: Manoela (não Manuela) em todos os documentos
- perfil-lider.md, POP de Qualidade OSID (.md e .docx) e Escala de Férias (.xlsx)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013f2XRhDo2k4tpqWLL7XirX
</commit_message>
<xml_diff>
--- a/meu-projeto/Escala-Ferias-OSID-CICAN-Dez26-Jan27.xlsx
+++ b/meu-projeto/Escala-Ferias-OSID-CICAN-Dez26-Jan27.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Manuela Carrera</t>
+          <t>Manoela Carrera</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -1119,7 +1119,7 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>3. Manuela Carrera não atua na assistência do CICAN — lá é só coordenadora. Por isso, sua coluna só permite OSID ou FÉRIAS.</t>
+          <t>3. Manoela Carrera não atua na assistência do CICAN — lá é só coordenadora. Por isso, sua coluna só permite OSID ou FÉRIAS.</t>
         </is>
       </c>
     </row>
@@ -1154,14 +1154,14 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>OSID: Manuela Carrera (coordenadora, com assistência), Éder Gerardo (subcoordenação), Ana Carolina Pondé, Laura, Juliana Azevedo, Tila Fortuna, Juliana Borges.</t>
+          <t>OSID: Manoela Carrera (coordenadora, com assistência), Éder Gerardo (subcoordenação), Ana Carolina Pondé, Laura, Juliana Azevedo, Tila Fortuna, Juliana Borges.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>CICAN: Éder Gerardo (subcoordenação), Ana Carolina Pondé, Laura, Juliana Azevedo. Manuela Carrera coordena, mas não entra na escala de assistência do CICAN. Nestor ainda não entra na escala — ingressará em breve.</t>
+          <t>CICAN: Éder Gerardo (subcoordenação), Ana Carolina Pondé, Laura, Juliana Azevedo. Manoela Carrera coordena, mas não entra na escala de assistência do CICAN. Nestor ainda não entra na escala — ingressará em breve.</t>
         </is>
       </c>
     </row>

</xml_diff>